<commit_message>
Fix downloaded files missing extensions and improve download handling
</commit_message>
<xml_diff>
--- a/output/provider_verification_output.xlsx
+++ b/output/provider_verification_output.xlsx
@@ -186,6 +186,26 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Credential and NPI Finder</author>
+  </authors>
+  <commentList>
+    <comment ref="AU3" authorId="0" shapeId="0">
+      <text>
+        <t>Entity mismatch — this is an Organization (Type 2: KYLE CORBIN, DC PA) NPI</t>
+      </text>
+    </comment>
+    <comment ref="AU10" authorId="0" shapeId="0">
+      <text>
+        <t>Entity mismatch — this is an Organization (Type 2: ADVANCED NEUROMODULATION SYSTEMS, INC.) NPI</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -477,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB20"/>
+  <dimension ref="A1:BG20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -487,12 +507,12 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
     <col width="59" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="53" customWidth="1" min="10" max="10"/>
     <col width="59" customWidth="1" min="11" max="11"/>
     <col width="29" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
     <col width="65" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="65" customWidth="1" min="16" max="16"/>
@@ -534,6 +554,11 @@
     <col width="14" customWidth="1" min="52" max="52"/>
     <col width="14" customWidth="1" min="53" max="53"/>
     <col width="14" customWidth="1" min="54" max="54"/>
+    <col width="25" customWidth="1" min="55" max="55"/>
+    <col width="31" customWidth="1" min="56" max="56"/>
+    <col width="23" customWidth="1" min="57" max="57"/>
+    <col width="19" customWidth="1" min="58" max="58"/>
+    <col width="65" customWidth="1" min="59" max="59"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -807,6 +832,31 @@
           <t>Unnamed: 53</t>
         </is>
       </c>
+      <c r="BC1" s="2" t="inlineStr">
+        <is>
+          <t>NPI Status</t>
+        </is>
+      </c>
+      <c r="BD1" s="2" t="inlineStr">
+        <is>
+          <t>NPI Entity Type</t>
+        </is>
+      </c>
+      <c r="BE1" s="2" t="inlineStr">
+        <is>
+          <t>NPI Validation</t>
+        </is>
+      </c>
+      <c r="BF1" s="2" t="inlineStr">
+        <is>
+          <t>Match Confidence</t>
+        </is>
+      </c>
+      <c r="BG1" s="2" t="inlineStr">
+        <is>
+          <t>Validation Notes</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -842,10 +892,14 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Unable to verify</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr"/>
+          <t>Credential not confirmed</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>https://npiregistry.cms.hhs.gov/provider-view/1649495409</t>
+        </is>
+      </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
           <t>1649495409</t>
@@ -864,7 +918,7 @@
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1649495409 | Credential could not be reliably verified.</t>
+          <t>Verified successfully</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr"/>
@@ -1011,6 +1065,31 @@
       <c r="AZ2" s="3" t="inlineStr"/>
       <c r="BA2" s="3" t="inlineStr"/>
       <c r="BB2" s="3" t="inlineStr"/>
+      <c r="BC2" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BD2" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE2" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BF2" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="BG2" s="3" t="inlineStr">
+        <is>
+          <t>Verified successfully</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -1046,7 +1125,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>D.C.</t>
+          <t>DC</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -1072,7 +1151,7 @@
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>PENDINGCPNAME is a provider name, but NPI column contains an Organization NPI (NPI-2: KYLE CORBIN, DC PA). | Provider NPI1: 1184909145</t>
+          <t>Entity mismatch — this is an Organization (Type 2: KYLE CORBIN, DC PA) NPI</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr"/>
@@ -1219,6 +1298,31 @@
       <c r="AZ3" s="3" t="inlineStr"/>
       <c r="BA3" s="3" t="inlineStr"/>
       <c r="BB3" s="3" t="inlineStr"/>
+      <c r="BC3" s="3" t="inlineStr">
+        <is>
+          <t>Entity Type Mismatch</t>
+        </is>
+      </c>
+      <c r="BD3" s="3" t="inlineStr">
+        <is>
+          <t>Type 2 — Organization</t>
+        </is>
+      </c>
+      <c r="BE3" s="3" t="inlineStr">
+        <is>
+          <t>Entity Type Mismatch</t>
+        </is>
+      </c>
+      <c r="BF3" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="BG3" s="3" t="inlineStr">
+        <is>
+          <t>Entity mismatch — this is an Organization (Type 2: KYLE CORBIN, DC PA) NPI</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -1254,33 +1358,25 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>M.D.</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>https://npiregistry.cms.hhs.gov/provider-view/1922856384</t>
-        </is>
-      </c>
+          <t>Credential not confirmed</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr"/>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>1922856384</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>https://npiregistry.cms.hhs.gov/provider-view/1922856384</t>
-        </is>
-      </c>
+          <t>Multiple possible matches — manual review required</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr"/>
       <c r="L4" s="3" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Requires Review</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1922856384</t>
+          <t>Multiple possible matches — manual review required</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr"/>
@@ -1415,6 +1511,31 @@
       <c r="AZ4" s="3" t="inlineStr"/>
       <c r="BA4" s="3" t="inlineStr"/>
       <c r="BB4" s="3" t="inlineStr"/>
+      <c r="BC4" s="3" t="inlineStr">
+        <is>
+          <t>Multiple Matches</t>
+        </is>
+      </c>
+      <c r="BD4" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE4" s="3" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="BF4" s="3" t="inlineStr">
+        <is>
+          <t>Manual Review</t>
+        </is>
+      </c>
+      <c r="BG4" s="3" t="inlineStr">
+        <is>
+          <t>Multiple possible matches — manual review required</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -1450,22 +1571,22 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>FNP-C</t>
+          <t>FNP</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>https://npiregistry.cms.hhs.gov/provider-view/1891321758</t>
+          <t>https://npiregistry.cms.hhs.gov/provider-view/1366476970</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>1891321758</t>
+          <t>1366476970</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>https://npiregistry.cms.hhs.gov/provider-view/1891321758</t>
+          <t>https://npiregistry.cms.hhs.gov/provider-view/1366476970</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr"/>
@@ -1476,7 +1597,7 @@
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1891321758</t>
+          <t>Verified successfully</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr"/>
@@ -1611,6 +1732,31 @@
       <c r="AZ5" s="3" t="inlineStr"/>
       <c r="BA5" s="3" t="inlineStr"/>
       <c r="BB5" s="3" t="inlineStr"/>
+      <c r="BC5" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BD5" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE5" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BF5" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="BG5" s="3" t="inlineStr">
+        <is>
+          <t>Verified successfully</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -1646,7 +1792,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>FNP-C</t>
+          <t>FNP</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -1672,7 +1818,7 @@
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1891321758</t>
+          <t>Verified successfully</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr"/>
@@ -1799,6 +1945,31 @@
       <c r="AZ6" s="3" t="inlineStr"/>
       <c r="BA6" s="3" t="inlineStr"/>
       <c r="BB6" s="3" t="inlineStr"/>
+      <c r="BC6" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BD6" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE6" s="3" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="BF6" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="BG6" s="3" t="inlineStr">
+        <is>
+          <t>Verified successfully</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -1860,7 +2031,7 @@
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1588313282</t>
+          <t>Verified successfully</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr"/>
@@ -1987,6 +2158,31 @@
       <c r="AZ7" s="3" t="inlineStr"/>
       <c r="BA7" s="3" t="inlineStr"/>
       <c r="BB7" s="3" t="inlineStr"/>
+      <c r="BC7" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BD7" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE7" s="3" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="BF7" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="BG7" s="3" t="inlineStr">
+        <is>
+          <t>Verified successfully</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -2048,7 +2244,7 @@
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1588313282</t>
+          <t>Verified successfully</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr"/>
@@ -2175,6 +2371,31 @@
       <c r="AZ8" s="3" t="inlineStr"/>
       <c r="BA8" s="3" t="inlineStr"/>
       <c r="BB8" s="3" t="inlineStr"/>
+      <c r="BC8" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BD8" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE8" s="3" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="BF8" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="BG8" s="3" t="inlineStr">
+        <is>
+          <t>Verified successfully</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -2236,7 +2457,7 @@
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1497722391</t>
+          <t>Verified successfully</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr"/>
@@ -2363,6 +2584,31 @@
       <c r="AZ9" s="3" t="inlineStr"/>
       <c r="BA9" s="3" t="inlineStr"/>
       <c r="BB9" s="3" t="inlineStr"/>
+      <c r="BC9" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BD9" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE9" s="3" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="BF9" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="BG9" s="3" t="inlineStr">
+        <is>
+          <t>Verified successfully</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -2424,7 +2670,7 @@
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>PENDINGCPNAME is a provider name, but NPI column contains an Organization NPI (NPI-2: ADVANCED NEUROMODULATION SYSTEMS, INC.). | Provider NPI1: 1356050694</t>
+          <t>Entity mismatch — this is an Organization (Type 2: ADVANCED NEUROMODULATION SYSTEMS, INC.) NPI</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr"/>
@@ -2555,6 +2801,31 @@
       <c r="AZ10" s="3" t="inlineStr"/>
       <c r="BA10" s="3" t="inlineStr"/>
       <c r="BB10" s="3" t="inlineStr"/>
+      <c r="BC10" s="3" t="inlineStr">
+        <is>
+          <t>Entity Type Mismatch</t>
+        </is>
+      </c>
+      <c r="BD10" s="3" t="inlineStr">
+        <is>
+          <t>Type 2 — Organization</t>
+        </is>
+      </c>
+      <c r="BE10" s="3" t="inlineStr">
+        <is>
+          <t>Entity Type Mismatch</t>
+        </is>
+      </c>
+      <c r="BF10" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="BG10" s="3" t="inlineStr">
+        <is>
+          <t>Entity mismatch — this is an Organization (Type 2: ADVANCED NEUROMODULATION SYSTEMS, INC.) NPI</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
@@ -2590,7 +2861,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>APRN-CNP</t>
+          <t>APRN</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -2616,7 +2887,7 @@
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1972257798</t>
+          <t>Verified successfully</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr"/>
@@ -2743,6 +3014,31 @@
       <c r="AZ11" s="3" t="inlineStr"/>
       <c r="BA11" s="3" t="inlineStr"/>
       <c r="BB11" s="3" t="inlineStr"/>
+      <c r="BC11" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BD11" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE11" s="3" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="BF11" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="BG11" s="3" t="inlineStr">
+        <is>
+          <t>Verified successfully</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
@@ -2778,29 +3074,25 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Unable to verify</t>
+          <t>Credential not confirmed</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr"/>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>1023512225</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>https://npiregistry.cms.hhs.gov/provider-view/1023512225</t>
-        </is>
-      </c>
+          <t>Multiple possible matches — manual review required</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr"/>
       <c r="L12" s="3" t="inlineStr"/>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Requires Review</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1023512225 | Credential could not be reliably verified.</t>
+          <t>Low confidence match — manual review required</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr"/>
@@ -2927,6 +3219,31 @@
       <c r="AZ12" s="3" t="inlineStr"/>
       <c r="BA12" s="3" t="inlineStr"/>
       <c r="BB12" s="3" t="inlineStr"/>
+      <c r="BC12" s="3" t="inlineStr">
+        <is>
+          <t>Manual Review Required</t>
+        </is>
+      </c>
+      <c r="BD12" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE12" s="3" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="BF12" s="3" t="inlineStr">
+        <is>
+          <t>Manual Review</t>
+        </is>
+      </c>
+      <c r="BG12" s="3" t="inlineStr">
+        <is>
+          <t>Low confidence match — manual review required</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -2988,7 +3305,7 @@
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1417679762</t>
+          <t>Verified successfully</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr"/>
@@ -3119,6 +3436,31 @@
       <c r="AZ13" s="3" t="inlineStr"/>
       <c r="BA13" s="3" t="inlineStr"/>
       <c r="BB13" s="3" t="inlineStr"/>
+      <c r="BC13" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BD13" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE13" s="3" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="BF13" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="BG13" s="3" t="inlineStr">
+        <is>
+          <t>Verified successfully</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -3180,7 +3522,7 @@
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1306816467</t>
+          <t>Verified successfully</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr"/>
@@ -3327,6 +3669,31 @@
       <c r="AZ14" s="3" t="inlineStr"/>
       <c r="BA14" s="3" t="inlineStr"/>
       <c r="BB14" s="3" t="inlineStr"/>
+      <c r="BC14" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BD14" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE14" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BF14" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="BG14" s="3" t="inlineStr">
+        <is>
+          <t>Verified successfully</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -3388,7 +3755,7 @@
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1063297083</t>
+          <t>Verified successfully</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr"/>
@@ -3535,6 +3902,31 @@
       <c r="AZ15" s="3" t="inlineStr"/>
       <c r="BA15" s="3" t="inlineStr"/>
       <c r="BB15" s="3" t="inlineStr"/>
+      <c r="BC15" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BD15" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE15" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BF15" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="BG15" s="3" t="inlineStr">
+        <is>
+          <t>Verified successfully</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -3570,33 +3962,25 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>BA</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>https://npiregistry.cms.hhs.gov/provider-view/1891827192</t>
-        </is>
-      </c>
+          <t>Credential not confirmed</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr"/>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>1891827192</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>https://npiregistry.cms.hhs.gov/provider-view/1891827192</t>
-        </is>
-      </c>
+          <t>Multiple possible matches — manual review required</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr"/>
       <c r="L16" s="3" t="inlineStr"/>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Requires Review</t>
         </is>
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1891827192</t>
+          <t>Multiple possible matches — manual review required</t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr"/>
@@ -3723,6 +4107,31 @@
       <c r="AZ16" s="3" t="inlineStr"/>
       <c r="BA16" s="3" t="inlineStr"/>
       <c r="BB16" s="3" t="inlineStr"/>
+      <c r="BC16" s="3" t="inlineStr">
+        <is>
+          <t>Multiple Matches</t>
+        </is>
+      </c>
+      <c r="BD16" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE16" s="3" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="BF16" s="3" t="inlineStr">
+        <is>
+          <t>Manual Review</t>
+        </is>
+      </c>
+      <c r="BG16" s="3" t="inlineStr">
+        <is>
+          <t>Multiple possible matches — manual review required</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -3758,7 +4167,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>M.D.</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -3784,7 +4193,7 @@
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1578523155</t>
+          <t>Verified successfully</t>
         </is>
       </c>
       <c r="O17" s="3" t="inlineStr"/>
@@ -3915,6 +4324,31 @@
       <c r="AZ17" s="3" t="inlineStr"/>
       <c r="BA17" s="3" t="inlineStr"/>
       <c r="BB17" s="3" t="inlineStr"/>
+      <c r="BC17" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BD17" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE17" s="3" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="BF17" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="BG17" s="3" t="inlineStr">
+        <is>
+          <t>Verified successfully</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
@@ -3953,21 +4387,13 @@
           <t>RN</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>https://npiregistry.cms.hhs.gov/provider-view/1487632329</t>
-        </is>
-      </c>
+      <c r="I18" s="3" t="inlineStr"/>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>1487632329</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>https://npiregistry.cms.hhs.gov/provider-view/1487632329</t>
-        </is>
-      </c>
+          <t>Multiple possible matches — manual review required</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr"/>
       <c r="L18" s="3" t="inlineStr"/>
       <c r="M18" s="3" t="inlineStr">
         <is>
@@ -3976,7 +4402,7 @@
       </c>
       <c r="N18" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1487632329</t>
+          <t>Multiple possible matches — manual review required</t>
         </is>
       </c>
       <c r="O18" s="3" t="inlineStr"/>
@@ -4103,6 +4529,31 @@
       <c r="AZ18" s="3" t="inlineStr"/>
       <c r="BA18" s="3" t="inlineStr"/>
       <c r="BB18" s="3" t="inlineStr"/>
+      <c r="BC18" s="3" t="inlineStr">
+        <is>
+          <t>Multiple Matches</t>
+        </is>
+      </c>
+      <c r="BD18" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE18" s="3" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="BF18" s="3" t="inlineStr">
+        <is>
+          <t>Manual Review</t>
+        </is>
+      </c>
+      <c r="BG18" s="3" t="inlineStr">
+        <is>
+          <t>Multiple possible matches — manual review required</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
@@ -4138,7 +4589,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>APNP</t>
+          <t>FNP</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -4164,7 +4615,7 @@
       </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1548701543</t>
+          <t>Verified successfully</t>
         </is>
       </c>
       <c r="O19" s="3" t="inlineStr"/>
@@ -4291,6 +4742,31 @@
       <c r="AZ19" s="3" t="inlineStr"/>
       <c r="BA19" s="3" t="inlineStr"/>
       <c r="BB19" s="3" t="inlineStr"/>
+      <c r="BC19" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BD19" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE19" s="3" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="BF19" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="BG19" s="3" t="inlineStr">
+        <is>
+          <t>Verified successfully</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
@@ -4352,7 +4828,7 @@
       </c>
       <c r="N20" s="3" t="inlineStr">
         <is>
-          <t>Provider NPI1: 1134840911</t>
+          <t>Verified successfully</t>
         </is>
       </c>
       <c r="O20" s="3" t="inlineStr"/>
@@ -4499,84 +4975,104 @@
       <c r="AZ20" s="3" t="inlineStr"/>
       <c r="BA20" s="3" t="inlineStr"/>
       <c r="BB20" s="3" t="inlineStr"/>
+      <c r="BC20" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BD20" s="3" t="inlineStr">
+        <is>
+          <t>Type 1 — Individual/Provider</t>
+        </is>
+      </c>
+      <c r="BE20" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="BF20" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="BG20" s="3" t="inlineStr">
+        <is>
+          <t>Verified successfully</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>